<commit_message>
Feature chinh sua thong tin ca nhan
</commit_message>
<xml_diff>
--- a/MoTaCongViec.xlsx
+++ b/MoTaCongViec.xlsx
@@ -4,10 +4,11 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="28260" windowHeight="13400"/>
+    <workbookView windowWidth="28260" windowHeight="13420"/>
   </bookViews>
   <sheets>
     <sheet name="Mô tả công việc" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -1415,4 +1416,15 @@
   <pageSetup paperSize="1" orientation="portrait"/>
   <headerFooter/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.8"/>
+  <sheetData/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
refactor: rename 'soNha' to 'diaChi' in event schema and related components
</commit_message>
<xml_diff>
--- a/MoTaCongViec.xlsx
+++ b/MoTaCongViec.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="29400" windowHeight="13420"/>
+    <workbookView windowWidth="29400" windowHeight="13400"/>
   </bookViews>
   <sheets>
     <sheet name="Mô tả công việc" sheetId="1" r:id="rId1"/>
@@ -809,7 +809,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -831,9 +831,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="58" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -1186,7 +1183,7 @@
       <c r="D1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="12" t="s">
+      <c r="E1" s="11" t="s">
         <v>4</v>
       </c>
     </row>
@@ -1228,7 +1225,7 @@
       <c r="A4" s="4">
         <v>3</v>
       </c>
-      <c r="B4" s="13" t="s">
+      <c r="B4" s="12" t="s">
         <v>13</v>
       </c>
       <c r="C4" s="9" t="s">
@@ -1245,7 +1242,7 @@
       <c r="A5" s="4">
         <v>4</v>
       </c>
-      <c r="B5" s="14" t="s">
+      <c r="B5" s="13" t="s">
         <v>16</v>
       </c>
       <c r="C5" s="9" t="s">
@@ -1285,7 +1282,7 @@
       <c r="C7" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="D7" s="10" t="s">
+      <c r="D7" s="9" t="s">
         <v>23</v>
       </c>
       <c r="E7" s="7" t="s">
@@ -1311,7 +1308,7 @@
       <c r="A9" s="4">
         <v>8</v>
       </c>
-      <c r="B9" s="14" t="s">
+      <c r="B9" s="13" t="s">
         <v>25</v>
       </c>
       <c r="C9" s="9" t="s">
@@ -1341,7 +1338,7 @@
       <c r="A11" s="4">
         <v>10</v>
       </c>
-      <c r="B11" s="11" t="s">
+      <c r="B11" s="10" t="s">
         <v>28</v>
       </c>
       <c r="C11" s="9" t="s">
@@ -1356,7 +1353,7 @@
       <c r="A12" s="4">
         <v>11</v>
       </c>
-      <c r="B12" s="11" t="s">
+      <c r="B12" s="10" t="s">
         <v>29</v>
       </c>
       <c r="C12" s="9" t="s">
@@ -1371,7 +1368,7 @@
       <c r="A13" s="4">
         <v>12</v>
       </c>
-      <c r="B13" s="15" t="s">
+      <c r="B13" s="14" t="s">
         <v>30</v>
       </c>
       <c r="C13" s="9" t="s">
@@ -1386,7 +1383,7 @@
       <c r="A14" s="4">
         <v>13</v>
       </c>
-      <c r="B14" s="13" t="s">
+      <c r="B14" s="12" t="s">
         <v>31</v>
       </c>
       <c r="C14" s="9" t="s">
@@ -1401,7 +1398,7 @@
       <c r="A15" s="4">
         <v>14</v>
       </c>
-      <c r="B15" s="11" t="s">
+      <c r="B15" s="10" t="s">
         <v>32</v>
       </c>
       <c r="C15" s="9" t="s">
@@ -1416,7 +1413,7 @@
       <c r="A16" s="4">
         <v>15</v>
       </c>
-      <c r="B16" s="11" t="s">
+      <c r="B16" s="10" t="s">
         <v>33</v>
       </c>
       <c r="C16" s="7" t="s">

</xml_diff>